<commit_message>
Ajusta a PCP e o Checklist aos casos de uso revisados e a 7 sprints
Ajustes apontados na apresentação da Iniciação (#21):

- PCP: backlog, priorização VRDC, APF e riscos passam a usar UC01 a
  UC12. UC03 reúne os antigos Iniciar, Calcular Previsão e Encerrar, com
  a maior nota VRDC de cada critério; as horas estimadas não mudam.
- Plano de entregas com 7 sprints, o número calculado na aba
  Planejamento (6,13 arredondado para cima), terminando em 20/11. A nota
  da aba Entregas registra que Construção e Transição ficam justas.
- Corrige notas que ainda citavam o plano de 8 sprints, o RI-12 e a
  estimativa de 728 h.
- Checklist: item 1 volta a Sim com o template do Documento de
  Requisitos; restaura as justificativas dos itens 16 e 17 (NA) e a
  observação do modelo no Astah, perdidas em 15/09. IAP de 100%.
</commit_message>
<xml_diff>
--- a/6.Gerenciamento de Projeto/CARREGAJA - Checklist de Projeto.xlsx
+++ b/6.Gerenciamento de Projeto/CARREGAJA - Checklist de Projeto.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{D1506729-BD29-4FDC-A8F6-3BD22061EEED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{204189F8-024C-49FA-A128-1306996FEC74}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{077A368B-FBA1-43EB-B3C8-DAD3BA2D068B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="666" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="960" yWindow="960" windowWidth="21600" windowHeight="11235" tabRatio="666" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Indicadores" sheetId="6" r:id="rId1"/>
@@ -713,7 +713,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="127">
   <si>
     <t>Ambiente</t>
   </si>
@@ -1057,9 +1057,6 @@
     <t>Foram realizados os testes de aceitação por parte do usuário final?</t>
   </si>
   <si>
-    <t>31/08/2026</t>
-  </si>
-  <si>
     <t>Henrique de Almeida Marangoni Inacio (Scrum Master)</t>
   </si>
   <si>
@@ -1075,10 +1072,28 @@
     <t>O Glossário é a subseção 1.3 do Visão, onde o template o posiciona. O SpinOff não prevê template autônomo para ele.</t>
   </si>
   <si>
-    <t>Não</t>
-  </si>
-  <si>
-    <t>Protótipo não produzido</t>
+    <t>26/09/2026</t>
+  </si>
+  <si>
+    <t>O Documento de Requisitos, não previsto no SpinOff, tem template próprio: 1.Requisitos/Template - Documento de Requisitos.dotx.</t>
+  </si>
+  <si>
+    <t>Visão reduzido a uma visão geral na versão 4.0, após a apresentação da Iniciação; o detalhamento passou ao Documento de Requisitos.</t>
+  </si>
+  <si>
+    <t>Modelo mantido em CARREGAJA - Modelos de Análise e Design.asta, no formato do Template - Modelos Analise e Design do SpinOff, com os dois atores, os doze casos de uso UC01–UC12, cada um com descrição, e as relações de inclusão.</t>
+  </si>
+  <si>
+    <t>Protótipo não produzido: é saída de Detalhar Requisitos, da Elaboração.</t>
+  </si>
+  <si>
+    <t>Não houve reunião de levantamento a registrar: o projeto não dispõe de cliente externo (RE-16).</t>
+  </si>
+  <si>
+    <t>Não se aplica pelo mesmo motivo do item 16 (RE-16).</t>
+  </si>
+  <si>
+    <t>Plano de entregas com 7 sprints, o número calculado na aba Planejamento da PCP (6,13, arredondado para cima).</t>
   </si>
 </sst>
 </file>
@@ -1709,7 +1724,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.96153846153846156</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -1941,7 +1956,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>1</c:v>
@@ -2167,7 +2182,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -7416,13 +7431,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="39" style="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18">
+    <row r="1" spans="1:2" ht="18.75">
       <c r="A1" s="55" t="s">
         <v>70</v>
       </c>
@@ -7442,7 +7457,7 @@
       </c>
       <c r="B3" s="18">
         <f>'Ver-Iniciação1'!$F$2</f>
-        <v>0.96153846153846156</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -7487,16 +7502,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E6B2C1B-A599-4159-99C1-DE703E343043}">
   <dimension ref="A1:R37"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="18.33203125" customWidth="1"/>
-    <col min="2" max="2" width="8.109375" customWidth="1"/>
-    <col min="3" max="3" width="17.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.88671875" customWidth="1"/>
-    <col min="5" max="5" width="6.44140625" customWidth="1"/>
-    <col min="6" max="6" width="6.88671875" customWidth="1"/>
-    <col min="14" max="14" width="13.109375" customWidth="1"/>
-    <col min="16" max="16" width="11.33203125" customWidth="1"/>
+    <col min="1" max="1" width="18.28515625" customWidth="1"/>
+    <col min="2" max="2" width="8.140625" customWidth="1"/>
+    <col min="3" max="3" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.85546875" customWidth="1"/>
+    <col min="5" max="5" width="6.42578125" customWidth="1"/>
+    <col min="6" max="6" width="6.85546875" customWidth="1"/>
+    <col min="14" max="14" width="13.140625" customWidth="1"/>
+    <col min="16" max="16" width="11.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -7537,7 +7552,7 @@
       </c>
       <c r="B2" s="22">
         <f>('Ver-Iniciação1'!$G$5/SUM('Ver-Iniciação1'!$G$5:'Ver-Iniciação1'!$J$5))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C2" s="22">
         <f>('Ver-Iniciação1'!$H$5/SUM('Ver-Iniciação1'!$G$5:'Ver-Iniciação1'!$J$5))</f>
@@ -7545,7 +7560,7 @@
       </c>
       <c r="D2" s="22">
         <f>('Ver-Iniciação1'!$I$5/SUM('Ver-Iniciação1'!$G$5:'Ver-Iniciação1'!$J$5))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2" s="22">
         <f>('Ver-Iniciação1'!$J$5/SUM('Ver-Iniciação1'!$G$5:'Ver-Iniciação1'!$J$5))</f>
@@ -8520,19 +8535,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:J41"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="1" max="1" width="5.6640625" customWidth="1"/>
-    <col min="2" max="2" width="7.33203125" style="4" customWidth="1"/>
-    <col min="3" max="3" width="76.109375" style="2" customWidth="1"/>
-    <col min="4" max="4" width="15.33203125" customWidth="1"/>
-    <col min="5" max="6" width="47.5546875" customWidth="1"/>
-    <col min="7" max="7" width="7.5546875" customWidth="1"/>
-    <col min="8" max="8" width="8.5546875" customWidth="1"/>
-    <col min="9" max="10" width="7.5546875" customWidth="1"/>
+    <col min="1" max="1" width="5.7109375" customWidth="1"/>
+    <col min="2" max="2" width="7.28515625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="76.140625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="15.28515625" customWidth="1"/>
+    <col min="5" max="6" width="47.5703125" customWidth="1"/>
+    <col min="7" max="7" width="7.5703125" customWidth="1"/>
+    <col min="8" max="8" width="8.5703125" customWidth="1"/>
+    <col min="9" max="10" width="7.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" ht="18">
       <c r="A1" s="46" t="s">
         <v>16</v>
       </c>
@@ -8552,7 +8567,7 @@
       </c>
       <c r="B2" s="47"/>
       <c r="C2" s="40" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="D2" s="53" t="s">
         <v>44</v>
@@ -8560,7 +8575,7 @@
       <c r="E2" s="54"/>
       <c r="F2" s="42">
         <f>COUNTIF(D5:D41,"Sim")/(COUNTA(D5:D41)-COUNTIF(D5:D41,"NA"))</f>
-        <v>0.96153846153846156</v>
+        <v>1</v>
       </c>
       <c r="G2" s="39"/>
       <c r="H2" s="39"/>
@@ -8573,7 +8588,7 @@
       </c>
       <c r="B3" s="47"/>
       <c r="C3" s="41" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D3" s="50" t="s">
         <v>43</v>
@@ -8585,7 +8600,7 @@
       <c r="I3" s="39"/>
       <c r="J3" s="39"/>
     </row>
-    <row r="4" spans="1:10" ht="28.8">
+    <row r="4" spans="1:10" ht="30">
       <c r="A4" s="25" t="s">
         <v>22</v>
       </c>
@@ -8609,7 +8624,7 @@
       <c r="I4" s="28"/>
       <c r="J4" s="28"/>
     </row>
-    <row r="5" spans="1:10" ht="14.4">
+    <row r="5" spans="1:10" ht="15">
       <c r="A5" s="48" t="s">
         <v>0</v>
       </c>
@@ -8622,7 +8637,7 @@
       <c r="F5" s="31"/>
       <c r="G5" s="28">
         <f>COUNTIF(D6,"Sim")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H5" s="28">
         <f>COUNTIF(D6,"Parcialmente")</f>
@@ -8630,14 +8645,14 @@
       </c>
       <c r="I5" s="28">
         <f>COUNTIF(D6,"Não")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" s="28">
         <f>COUNTIF(D6,"NA")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="14.4">
+    <row r="6" spans="1:10" ht="60">
       <c r="A6" s="49"/>
       <c r="B6" s="32">
         <v>1</v>
@@ -8646,16 +8661,18 @@
         <v>33</v>
       </c>
       <c r="D6" s="34" t="s">
+        <v>115</v>
+      </c>
+      <c r="E6" s="33"/>
+      <c r="F6" s="33" t="s">
         <v>120</v>
       </c>
-      <c r="E6" s="33"/>
-      <c r="F6" s="33"/>
       <c r="G6" s="28"/>
       <c r="H6" s="28"/>
       <c r="I6" s="28"/>
       <c r="J6" s="28"/>
     </row>
-    <row r="7" spans="1:10" ht="14.4">
+    <row r="7" spans="1:10" ht="15">
       <c r="A7" s="48" t="s">
         <v>17</v>
       </c>
@@ -8683,7 +8700,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="28.8">
+    <row r="8" spans="1:10" ht="30">
       <c r="A8" s="45"/>
       <c r="B8" s="35">
         <v>2</v>
@@ -8692,7 +8709,7 @@
         <v>72</v>
       </c>
       <c r="D8" s="34" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E8" s="33"/>
       <c r="F8" s="33"/>
@@ -8701,7 +8718,7 @@
       <c r="I8" s="28"/>
       <c r="J8" s="28"/>
     </row>
-    <row r="9" spans="1:10" ht="14.4">
+    <row r="9" spans="1:10" ht="15">
       <c r="A9" s="45"/>
       <c r="B9" s="32">
         <v>3</v>
@@ -8710,7 +8727,7 @@
         <v>31</v>
       </c>
       <c r="D9" s="34" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E9" s="33"/>
       <c r="F9" s="33"/>
@@ -8719,7 +8736,7 @@
       <c r="I9" s="28"/>
       <c r="J9" s="28"/>
     </row>
-    <row r="10" spans="1:10" ht="14.4">
+    <row r="10" spans="1:10" ht="15">
       <c r="A10" s="45"/>
       <c r="B10" s="32">
         <v>4</v>
@@ -8728,7 +8745,7 @@
         <v>77</v>
       </c>
       <c r="D10" s="34" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E10" s="33"/>
       <c r="F10" s="33"/>
@@ -8737,7 +8754,7 @@
       <c r="I10" s="28"/>
       <c r="J10" s="28"/>
     </row>
-    <row r="11" spans="1:10" s="1" customFormat="1" ht="14.4">
+    <row r="11" spans="1:10" s="1" customFormat="1" ht="45">
       <c r="A11" s="45"/>
       <c r="B11" s="32">
         <v>5</v>
@@ -8746,16 +8763,18 @@
         <v>32</v>
       </c>
       <c r="D11" s="34" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E11" s="33"/>
-      <c r="F11" s="33"/>
+      <c r="F11" s="33" t="s">
+        <v>121</v>
+      </c>
       <c r="G11" s="37"/>
       <c r="H11" s="37"/>
       <c r="I11" s="37"/>
       <c r="J11" s="37"/>
     </row>
-    <row r="12" spans="1:10" ht="28.8">
+    <row r="12" spans="1:10" ht="30">
       <c r="A12" s="45"/>
       <c r="B12" s="32">
         <v>6</v>
@@ -8764,7 +8783,7 @@
         <v>40</v>
       </c>
       <c r="D12" s="34" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E12" s="33"/>
       <c r="F12" s="33"/>
@@ -8773,7 +8792,7 @@
       <c r="I12" s="28"/>
       <c r="J12" s="28"/>
     </row>
-    <row r="13" spans="1:10" ht="14.4">
+    <row r="13" spans="1:10" ht="15">
       <c r="A13" s="45"/>
       <c r="B13" s="29"/>
       <c r="C13" s="30" t="s">
@@ -8799,7 +8818,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="28.8">
+    <row r="14" spans="1:10" ht="75">
       <c r="A14" s="45"/>
       <c r="B14" s="38">
         <v>7</v>
@@ -8808,16 +8827,18 @@
         <v>72</v>
       </c>
       <c r="D14" s="34" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E14" s="33"/>
-      <c r="F14" s="33"/>
+      <c r="F14" s="33" t="s">
+        <v>122</v>
+      </c>
       <c r="G14" s="28"/>
       <c r="H14" s="28"/>
       <c r="I14" s="28"/>
       <c r="J14" s="28"/>
     </row>
-    <row r="15" spans="1:10" s="1" customFormat="1" ht="28.8">
+    <row r="15" spans="1:10" s="1" customFormat="1" ht="30">
       <c r="A15" s="45"/>
       <c r="B15" s="32">
         <v>8</v>
@@ -8826,7 +8847,7 @@
         <v>34</v>
       </c>
       <c r="D15" s="34" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E15" s="33"/>
       <c r="F15" s="33"/>
@@ -8835,7 +8856,7 @@
       <c r="I15" s="37"/>
       <c r="J15" s="37"/>
     </row>
-    <row r="16" spans="1:10" s="1" customFormat="1" ht="28.8">
+    <row r="16" spans="1:10" s="1" customFormat="1" ht="30">
       <c r="A16" s="45"/>
       <c r="B16" s="32">
         <v>9</v>
@@ -8844,7 +8865,7 @@
         <v>79</v>
       </c>
       <c r="D16" s="34" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E16" s="33"/>
       <c r="F16" s="33"/>
@@ -8853,7 +8874,7 @@
       <c r="I16" s="37"/>
       <c r="J16" s="37"/>
     </row>
-    <row r="17" spans="1:10" s="1" customFormat="1" ht="28.8">
+    <row r="17" spans="1:10" s="1" customFormat="1" ht="30">
       <c r="A17" s="45"/>
       <c r="B17" s="38">
         <v>10</v>
@@ -8862,10 +8883,10 @@
         <v>76</v>
       </c>
       <c r="D17" s="34" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E17" s="33" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F17" s="33"/>
       <c r="G17" s="37"/>
@@ -8873,7 +8894,7 @@
       <c r="I17" s="37"/>
       <c r="J17" s="37"/>
     </row>
-    <row r="18" spans="1:10" s="1" customFormat="1" ht="28.8">
+    <row r="18" spans="1:10" s="1" customFormat="1" ht="30">
       <c r="A18" s="45"/>
       <c r="B18" s="32">
         <v>11</v>
@@ -8882,18 +8903,18 @@
         <v>75</v>
       </c>
       <c r="D18" s="34" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E18" s="33"/>
       <c r="F18" s="33" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G18" s="37"/>
       <c r="H18" s="37"/>
       <c r="I18" s="37"/>
       <c r="J18" s="37"/>
     </row>
-    <row r="19" spans="1:10" ht="14.4">
+    <row r="19" spans="1:10" ht="15">
       <c r="A19" s="45"/>
       <c r="B19" s="29"/>
       <c r="C19" s="30" t="s">
@@ -8919,7 +8940,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="28.8">
+    <row r="20" spans="1:10" ht="30">
       <c r="A20" s="45"/>
       <c r="B20" s="38">
         <v>12</v>
@@ -8928,7 +8949,7 @@
         <v>78</v>
       </c>
       <c r="D20" s="34" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E20" s="33"/>
       <c r="F20" s="33"/>
@@ -8937,7 +8958,7 @@
       <c r="I20" s="28"/>
       <c r="J20" s="28"/>
     </row>
-    <row r="21" spans="1:10" ht="28.8">
+    <row r="21" spans="1:10" ht="45">
       <c r="A21" s="45"/>
       <c r="B21" s="32">
         <v>13</v>
@@ -8946,7 +8967,7 @@
         <v>80</v>
       </c>
       <c r="D21" s="34" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E21" s="33"/>
       <c r="F21" s="33"/>
@@ -8955,7 +8976,7 @@
       <c r="I21" s="28"/>
       <c r="J21" s="28"/>
     </row>
-    <row r="22" spans="1:10" ht="14.4">
+    <row r="22" spans="1:10" ht="15">
       <c r="A22" s="45"/>
       <c r="B22" s="29"/>
       <c r="C22" s="30" t="s">
@@ -8981,7 +9002,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="43.2">
+    <row r="23" spans="1:10" ht="45">
       <c r="A23" s="45"/>
       <c r="B23" s="38">
         <v>14</v>
@@ -8990,18 +9011,18 @@
         <v>72</v>
       </c>
       <c r="D23" s="34" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E23" s="33"/>
       <c r="F23" s="33" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G23" s="28"/>
       <c r="H23" s="28"/>
       <c r="I23" s="28"/>
       <c r="J23" s="28"/>
     </row>
-    <row r="24" spans="1:10" ht="14.4">
+    <row r="24" spans="1:10" ht="15">
       <c r="A24" s="45"/>
       <c r="B24" s="32">
         <v>15</v>
@@ -9010,7 +9031,7 @@
         <v>35</v>
       </c>
       <c r="D24" s="34" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E24" s="33"/>
       <c r="F24" s="33"/>
@@ -9019,7 +9040,7 @@
       <c r="I24" s="28"/>
       <c r="J24" s="28"/>
     </row>
-    <row r="25" spans="1:10" ht="14.4">
+    <row r="25" spans="1:10" ht="15">
       <c r="A25" s="45"/>
       <c r="B25" s="29"/>
       <c r="C25" s="30" t="s">
@@ -9045,7 +9066,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="28.8">
+    <row r="26" spans="1:10" ht="30">
       <c r="A26" s="45"/>
       <c r="B26" s="38">
         <v>16</v>
@@ -9054,16 +9075,18 @@
         <v>72</v>
       </c>
       <c r="D26" s="34" t="s">
-        <v>117</v>
-      </c>
-      <c r="E26" s="33"/>
+        <v>116</v>
+      </c>
+      <c r="E26" s="33" t="s">
+        <v>124</v>
+      </c>
       <c r="F26" s="33"/>
       <c r="G26" s="28"/>
       <c r="H26" s="28"/>
       <c r="I26" s="28"/>
       <c r="J26" s="28"/>
     </row>
-    <row r="27" spans="1:10" ht="14.4">
+    <row r="27" spans="1:10" ht="30">
       <c r="A27" s="45"/>
       <c r="B27" s="32">
         <v>17</v>
@@ -9072,16 +9095,18 @@
         <v>37</v>
       </c>
       <c r="D27" s="34" t="s">
-        <v>117</v>
-      </c>
-      <c r="E27" s="33"/>
+        <v>116</v>
+      </c>
+      <c r="E27" s="33" t="s">
+        <v>125</v>
+      </c>
       <c r="F27" s="33"/>
       <c r="G27" s="28"/>
       <c r="H27" s="28"/>
       <c r="I27" s="28"/>
       <c r="J27" s="28"/>
     </row>
-    <row r="28" spans="1:10" ht="14.4">
+    <row r="28" spans="1:10" ht="15">
       <c r="A28" s="45"/>
       <c r="B28" s="29"/>
       <c r="C28" s="30" t="s">
@@ -9107,7 +9132,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="28.8">
+    <row r="29" spans="1:10" ht="30">
       <c r="A29" s="45"/>
       <c r="B29" s="38">
         <v>21</v>
@@ -9116,7 +9141,7 @@
         <v>72</v>
       </c>
       <c r="D29" s="34" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E29" s="33"/>
       <c r="F29" s="33"/>
@@ -9125,7 +9150,7 @@
       <c r="I29" s="28"/>
       <c r="J29" s="28"/>
     </row>
-    <row r="30" spans="1:10" ht="14.4">
+    <row r="30" spans="1:10" ht="15">
       <c r="A30" s="45"/>
       <c r="B30" s="32">
         <v>22</v>
@@ -9134,7 +9159,7 @@
         <v>41</v>
       </c>
       <c r="D30" s="34" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E30" s="33"/>
       <c r="F30" s="33"/>
@@ -9143,7 +9168,7 @@
       <c r="I30" s="28"/>
       <c r="J30" s="28"/>
     </row>
-    <row r="31" spans="1:10" ht="14.4">
+    <row r="31" spans="1:10" ht="15">
       <c r="A31" s="45"/>
       <c r="B31" s="32">
         <v>23</v>
@@ -9152,7 +9177,7 @@
         <v>86</v>
       </c>
       <c r="D31" s="34" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E31" s="33"/>
       <c r="F31" s="33"/>
@@ -9161,7 +9186,7 @@
       <c r="I31" s="28"/>
       <c r="J31" s="28"/>
     </row>
-    <row r="32" spans="1:10" ht="14.4">
+    <row r="32" spans="1:10" ht="15">
       <c r="A32" s="45"/>
       <c r="B32" s="32">
         <v>24</v>
@@ -9170,7 +9195,7 @@
         <v>82</v>
       </c>
       <c r="D32" s="34" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E32" s="33"/>
       <c r="F32" s="33"/>
@@ -9179,7 +9204,7 @@
       <c r="I32" s="28"/>
       <c r="J32" s="28"/>
     </row>
-    <row r="33" spans="1:10" ht="14.4">
+    <row r="33" spans="1:10" ht="15">
       <c r="A33" s="45"/>
       <c r="B33" s="32">
         <v>25</v>
@@ -9188,7 +9213,7 @@
         <v>83</v>
       </c>
       <c r="D33" s="34" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E33" s="33"/>
       <c r="F33" s="33"/>
@@ -9197,7 +9222,7 @@
       <c r="I33" s="28"/>
       <c r="J33" s="28"/>
     </row>
-    <row r="34" spans="1:10" ht="28.8">
+    <row r="34" spans="1:10" ht="45">
       <c r="A34" s="45"/>
       <c r="B34" s="32">
         <v>26</v>
@@ -9206,16 +9231,18 @@
         <v>87</v>
       </c>
       <c r="D34" s="34" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E34" s="28"/>
-      <c r="F34" s="33"/>
+      <c r="F34" s="33" t="s">
+        <v>126</v>
+      </c>
       <c r="G34" s="28"/>
       <c r="H34" s="28"/>
       <c r="I34" s="28"/>
       <c r="J34" s="28"/>
     </row>
-    <row r="35" spans="1:10" ht="28.8">
+    <row r="35" spans="1:10" ht="30">
       <c r="A35" s="45"/>
       <c r="B35" s="32">
         <v>27</v>
@@ -9224,7 +9251,7 @@
         <v>84</v>
       </c>
       <c r="D35" s="34" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E35" s="33"/>
       <c r="F35" s="33"/>
@@ -9233,7 +9260,7 @@
       <c r="I35" s="28"/>
       <c r="J35" s="28"/>
     </row>
-    <row r="36" spans="1:10" ht="28.8">
+    <row r="36" spans="1:10" ht="30">
       <c r="A36" s="45"/>
       <c r="B36" s="32">
         <v>28</v>
@@ -9242,18 +9269,18 @@
         <v>85</v>
       </c>
       <c r="D36" s="33" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E36" s="33"/>
       <c r="F36" s="33" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G36" s="28"/>
       <c r="H36" s="28"/>
       <c r="I36" s="28"/>
       <c r="J36" s="28"/>
     </row>
-    <row r="37" spans="1:10" ht="14.4">
+    <row r="37" spans="1:10" ht="15">
       <c r="A37" s="43" t="s">
         <v>30</v>
       </c>
@@ -9281,7 +9308,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="28.8">
+    <row r="38" spans="1:10" ht="30">
       <c r="A38" s="44"/>
       <c r="B38" s="38">
         <v>30</v>
@@ -9290,7 +9317,7 @@
         <v>73</v>
       </c>
       <c r="D38" s="34" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E38" s="33"/>
       <c r="F38" s="33"/>
@@ -9299,7 +9326,7 @@
       <c r="I38" s="28"/>
       <c r="J38" s="28"/>
     </row>
-    <row r="39" spans="1:10" ht="28.8">
+    <row r="39" spans="1:10" ht="30">
       <c r="A39" s="44"/>
       <c r="B39" s="32">
         <v>31</v>
@@ -9308,7 +9335,7 @@
         <v>38</v>
       </c>
       <c r="D39" s="34" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E39" s="33"/>
       <c r="F39" s="33"/>
@@ -9317,7 +9344,7 @@
       <c r="I39" s="28"/>
       <c r="J39" s="28"/>
     </row>
-    <row r="40" spans="1:10" ht="14.4">
+    <row r="40" spans="1:10" ht="15">
       <c r="A40" s="44"/>
       <c r="B40" s="32">
         <v>32</v>
@@ -9326,7 +9353,7 @@
         <v>39</v>
       </c>
       <c r="D40" s="34" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E40" s="33"/>
       <c r="F40" s="33"/>
@@ -9335,7 +9362,7 @@
       <c r="I40" s="28"/>
       <c r="J40" s="28"/>
     </row>
-    <row r="41" spans="1:10" ht="28.8">
+    <row r="41" spans="1:10" ht="30">
       <c r="A41" s="44"/>
       <c r="B41" s="32">
         <v>33</v>
@@ -9344,7 +9371,7 @@
         <v>42</v>
       </c>
       <c r="D41" s="34" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E41" s="33"/>
       <c r="F41" s="33"/>
@@ -9379,14 +9406,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:J41"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="1" max="1" width="21.109375" customWidth="1"/>
-    <col min="2" max="2" width="5.33203125" style="4" customWidth="1"/>
+    <col min="1" max="1" width="21.140625" customWidth="1"/>
+    <col min="2" max="2" width="5.28515625" style="4" customWidth="1"/>
     <col min="3" max="3" width="68" style="2" customWidth="1"/>
-    <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="29.6640625" customWidth="1"/>
-    <col min="6" max="6" width="32.6640625" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.7109375" customWidth="1"/>
+    <col min="6" max="6" width="32.7109375" customWidth="1"/>
     <col min="7" max="10" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -9415,7 +9442,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="15" thickBot="1">
+    <row r="3" spans="1:10" ht="15.75" thickBot="1">
       <c r="A3" s="62" t="s">
         <v>26</v>
       </c>
@@ -9427,7 +9454,7 @@
       <c r="E3" s="66"/>
       <c r="F3" s="67"/>
     </row>
-    <row r="4" spans="1:10" ht="14.4">
+    <row r="4" spans="1:10" ht="15">
       <c r="A4" s="6" t="s">
         <v>22</v>
       </c>
@@ -9459,7 +9486,7 @@
       <c r="E5" s="12"/>
       <c r="F5" s="12"/>
     </row>
-    <row r="6" spans="1:10" ht="14.4">
+    <row r="6" spans="1:10" ht="15">
       <c r="A6" s="59"/>
       <c r="B6" s="5">
         <v>1</v>
@@ -9487,7 +9514,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="14.4">
+    <row r="7" spans="1:10" ht="15">
       <c r="A7" s="59"/>
       <c r="B7" s="9"/>
       <c r="C7" s="10" t="s">
@@ -9497,7 +9524,7 @@
       <c r="E7" s="12"/>
       <c r="F7" s="12"/>
     </row>
-    <row r="8" spans="1:10" s="1" customFormat="1" ht="28.8">
+    <row r="8" spans="1:10" s="1" customFormat="1" ht="30">
       <c r="A8" s="59"/>
       <c r="B8" s="5">
         <v>2</v>
@@ -9525,7 +9552,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" s="1" customFormat="1" ht="28.8">
+    <row r="9" spans="1:10" s="1" customFormat="1" ht="30">
       <c r="A9" s="59"/>
       <c r="B9" s="5">
         <v>3</v>
@@ -9541,7 +9568,7 @@
       <c r="I9"/>
       <c r="J9"/>
     </row>
-    <row r="10" spans="1:10" ht="14.4">
+    <row r="10" spans="1:10" ht="15">
       <c r="A10" s="59"/>
       <c r="B10" s="9"/>
       <c r="C10" s="10" t="s">
@@ -9551,7 +9578,7 @@
       <c r="E10" s="12"/>
       <c r="F10" s="12"/>
     </row>
-    <row r="11" spans="1:10" ht="28.8">
+    <row r="11" spans="1:10" ht="30">
       <c r="A11" s="59"/>
       <c r="B11" s="20">
         <v>4</v>
@@ -9579,7 +9606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="28.8">
+    <row r="12" spans="1:10" ht="30">
       <c r="A12" s="59"/>
       <c r="B12" s="20">
         <v>5</v>
@@ -9591,7 +9618,7 @@
       <c r="E12" s="8"/>
       <c r="F12" s="8"/>
     </row>
-    <row r="13" spans="1:10" ht="14.4">
+    <row r="13" spans="1:10" ht="30">
       <c r="A13" s="59"/>
       <c r="B13" s="5">
         <v>6</v>
@@ -9603,7 +9630,7 @@
       <c r="E13" s="8"/>
       <c r="F13" s="8"/>
     </row>
-    <row r="14" spans="1:10" ht="28.8">
+    <row r="14" spans="1:10" ht="30">
       <c r="A14" s="59"/>
       <c r="B14" s="5">
         <v>7</v>
@@ -9615,7 +9642,7 @@
       <c r="E14" s="8"/>
       <c r="F14" s="8"/>
     </row>
-    <row r="15" spans="1:10" ht="14.4">
+    <row r="15" spans="1:10" ht="15">
       <c r="A15" s="59"/>
       <c r="B15" s="9"/>
       <c r="C15" s="10" t="s">
@@ -9625,7 +9652,7 @@
       <c r="E15" s="12"/>
       <c r="F15" s="12"/>
     </row>
-    <row r="16" spans="1:10" ht="14.4">
+    <row r="16" spans="1:10" ht="15">
       <c r="A16" s="59"/>
       <c r="B16" s="5">
         <v>7</v>
@@ -9665,7 +9692,7 @@
       <c r="E17" s="12"/>
       <c r="F17" s="12"/>
     </row>
-    <row r="18" spans="1:10" ht="28.8">
+    <row r="18" spans="1:10" ht="30">
       <c r="A18" s="59"/>
       <c r="B18" s="5">
         <v>9</v>
@@ -9693,7 +9720,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="28.8">
+    <row r="19" spans="1:10" ht="30">
       <c r="A19" s="59"/>
       <c r="B19" s="20">
         <v>10</v>
@@ -9705,7 +9732,7 @@
       <c r="E19" s="8"/>
       <c r="F19" s="8"/>
     </row>
-    <row r="20" spans="1:10" s="1" customFormat="1" ht="28.8">
+    <row r="20" spans="1:10" s="1" customFormat="1" ht="30">
       <c r="A20" s="59"/>
       <c r="B20" s="5">
         <v>11</v>
@@ -9717,7 +9744,7 @@
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
     </row>
-    <row r="21" spans="1:10" ht="28.8">
+    <row r="21" spans="1:10" ht="45">
       <c r="A21" s="59"/>
       <c r="B21" s="5">
         <v>12</v>
@@ -9729,7 +9756,7 @@
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
     </row>
-    <row r="22" spans="1:10" ht="14.4">
+    <row r="22" spans="1:10" ht="15">
       <c r="A22" s="58" t="s">
         <v>19</v>
       </c>
@@ -9741,7 +9768,7 @@
       <c r="E22" s="12"/>
       <c r="F22" s="12"/>
     </row>
-    <row r="23" spans="1:10" ht="28.8">
+    <row r="23" spans="1:10" ht="30">
       <c r="A23" s="59"/>
       <c r="B23" s="5">
         <v>17</v>
@@ -9769,7 +9796,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="28.8">
+    <row r="24" spans="1:10" ht="30">
       <c r="A24" s="59"/>
       <c r="B24" s="5">
         <v>18</v>
@@ -9781,7 +9808,7 @@
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
     </row>
-    <row r="25" spans="1:10" ht="28.8">
+    <row r="25" spans="1:10" ht="30">
       <c r="A25" s="59"/>
       <c r="B25" s="5">
         <v>19</v>
@@ -9793,7 +9820,7 @@
       <c r="E25" s="8"/>
       <c r="F25" s="8"/>
     </row>
-    <row r="26" spans="1:10" ht="14.4">
+    <row r="26" spans="1:10" ht="15">
       <c r="A26" s="59"/>
       <c r="B26" s="5">
         <v>21</v>
@@ -9805,7 +9832,7 @@
       <c r="E26" s="8"/>
       <c r="F26" s="8"/>
     </row>
-    <row r="27" spans="1:10" ht="14.4">
+    <row r="27" spans="1:10" ht="15">
       <c r="A27" s="59"/>
       <c r="B27" s="5">
         <v>22</v>
@@ -9817,7 +9844,7 @@
       <c r="E27" s="8"/>
       <c r="F27" s="8"/>
     </row>
-    <row r="28" spans="1:10" ht="14.4">
+    <row r="28" spans="1:10" ht="15">
       <c r="A28" s="60" t="s">
         <v>11</v>
       </c>
@@ -9829,7 +9856,7 @@
       <c r="E28" s="12"/>
       <c r="F28" s="12"/>
     </row>
-    <row r="29" spans="1:10" ht="14.4">
+    <row r="29" spans="1:10" ht="15">
       <c r="A29" s="60"/>
       <c r="B29" s="5">
         <v>23</v>
@@ -9857,7 +9884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="14.4">
+    <row r="30" spans="1:10" ht="15">
       <c r="A30" s="60"/>
       <c r="B30" s="5">
         <v>24</v>
@@ -9869,7 +9896,7 @@
       <c r="E30" s="8"/>
       <c r="F30" s="8"/>
     </row>
-    <row r="31" spans="1:10" ht="28.8">
+    <row r="31" spans="1:10" ht="30">
       <c r="A31" s="60"/>
       <c r="B31" s="5">
         <v>25</v>
@@ -9881,7 +9908,7 @@
       <c r="E31" s="8"/>
       <c r="F31" s="8"/>
     </row>
-    <row r="32" spans="1:10" ht="14.4">
+    <row r="32" spans="1:10" ht="15">
       <c r="A32" s="60"/>
       <c r="B32" s="5">
         <v>26</v>
@@ -9893,7 +9920,7 @@
       <c r="E32" s="8"/>
       <c r="F32" s="8"/>
     </row>
-    <row r="33" spans="1:10" ht="14.4">
+    <row r="33" spans="1:10" ht="15">
       <c r="A33" s="60"/>
       <c r="B33" s="5">
         <v>27</v>
@@ -9905,7 +9932,7 @@
       <c r="E33" s="8"/>
       <c r="F33" s="8"/>
     </row>
-    <row r="34" spans="1:10" ht="14.4">
+    <row r="34" spans="1:10" ht="15">
       <c r="A34" s="60"/>
       <c r="B34" s="5">
         <v>28</v>
@@ -9929,7 +9956,7 @@
       <c r="E35" s="12"/>
       <c r="F35" s="12"/>
     </row>
-    <row r="36" spans="1:10" ht="28.8">
+    <row r="36" spans="1:10" ht="30">
       <c r="A36" s="57"/>
       <c r="B36" s="5">
         <v>29</v>
@@ -9957,7 +9984,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="14.4">
+    <row r="37" spans="1:10" ht="15">
       <c r="A37" s="57"/>
       <c r="B37" s="5">
         <v>30</v>
@@ -9969,7 +9996,7 @@
       <c r="E37" s="8"/>
       <c r="F37" s="8"/>
     </row>
-    <row r="38" spans="1:10" ht="28.8">
+    <row r="38" spans="1:10" ht="30">
       <c r="A38" s="57"/>
       <c r="B38" s="5">
         <v>31</v>
@@ -9981,7 +10008,7 @@
       <c r="E38" s="8"/>
       <c r="F38" s="8"/>
     </row>
-    <row r="39" spans="1:10" ht="14.4">
+    <row r="39" spans="1:10" ht="15">
       <c r="A39" s="57"/>
       <c r="B39" s="9"/>
       <c r="C39" s="10" t="s">
@@ -9991,7 +10018,7 @@
       <c r="E39" s="12"/>
       <c r="F39" s="12"/>
     </row>
-    <row r="40" spans="1:10" ht="14.4">
+    <row r="40" spans="1:10" ht="15">
       <c r="A40" s="57"/>
       <c r="B40" s="5">
         <v>32</v>
@@ -10019,7 +10046,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:10" ht="14.4">
+    <row r="41" spans="1:10" ht="15">
       <c r="A41" s="57"/>
       <c r="B41" s="5">
         <v>33</v>
@@ -10060,15 +10087,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:J57"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="1" max="1" width="21.109375" customWidth="1"/>
-    <col min="2" max="2" width="5.33203125" style="4" customWidth="1"/>
-    <col min="3" max="3" width="71.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="29.6640625" customWidth="1"/>
-    <col min="6" max="6" width="32.6640625" customWidth="1"/>
-    <col min="7" max="10" width="9.109375" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="21.140625" customWidth="1"/>
+    <col min="2" max="2" width="5.28515625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="71.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.7109375" customWidth="1"/>
+    <col min="6" max="6" width="32.7109375" customWidth="1"/>
+    <col min="7" max="10" width="9.140625" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="19.5" customHeight="1">
@@ -10096,7 +10123,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="15" thickBot="1">
+    <row r="3" spans="1:10" ht="15.75" thickBot="1">
       <c r="A3" s="62" t="s">
         <v>26</v>
       </c>
@@ -10108,7 +10135,7 @@
       <c r="E3" s="66"/>
       <c r="F3" s="67"/>
     </row>
-    <row r="4" spans="1:10" ht="14.4">
+    <row r="4" spans="1:10" ht="15">
       <c r="A4" s="6" t="s">
         <v>22</v>
       </c>
@@ -10140,7 +10167,7 @@
       <c r="E5" s="12"/>
       <c r="F5" s="12"/>
     </row>
-    <row r="6" spans="1:10" ht="14.4">
+    <row r="6" spans="1:10" ht="15">
       <c r="A6" s="59"/>
       <c r="B6" s="5">
         <v>1</v>
@@ -10168,7 +10195,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="14.4">
+    <row r="7" spans="1:10" ht="15">
       <c r="A7" s="59"/>
       <c r="B7" s="9"/>
       <c r="C7" s="10" t="s">
@@ -10178,7 +10205,7 @@
       <c r="E7" s="12"/>
       <c r="F7" s="12"/>
     </row>
-    <row r="8" spans="1:10" s="1" customFormat="1" ht="28.8">
+    <row r="8" spans="1:10" s="1" customFormat="1" ht="30">
       <c r="A8" s="59"/>
       <c r="B8" s="5">
         <v>2</v>
@@ -10206,7 +10233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="14.4">
+    <row r="9" spans="1:10" ht="15">
       <c r="A9" s="59"/>
       <c r="B9" s="9"/>
       <c r="C9" s="10" t="s">
@@ -10216,7 +10243,7 @@
       <c r="E9" s="12"/>
       <c r="F9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="28.8">
+    <row r="10" spans="1:10" ht="30">
       <c r="A10" s="59"/>
       <c r="B10" s="5">
         <v>3</v>
@@ -10244,7 +10271,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="28.8">
+    <row r="11" spans="1:10" ht="30">
       <c r="A11" s="59"/>
       <c r="B11" s="5">
         <v>4</v>
@@ -10268,7 +10295,7 @@
       <c r="E12" s="8"/>
       <c r="F12" s="8"/>
     </row>
-    <row r="13" spans="1:10" ht="14.4">
+    <row r="13" spans="1:10" ht="15">
       <c r="A13" s="59"/>
       <c r="B13" s="9"/>
       <c r="C13" s="10" t="s">
@@ -10278,7 +10305,7 @@
       <c r="E13" s="12"/>
       <c r="F13" s="12"/>
     </row>
-    <row r="14" spans="1:10" ht="14.4">
+    <row r="14" spans="1:10" ht="15">
       <c r="A14" s="59"/>
       <c r="B14" s="5">
         <v>6</v>
@@ -10318,7 +10345,7 @@
       <c r="E15" s="12"/>
       <c r="F15" s="12"/>
     </row>
-    <row r="16" spans="1:10" ht="14.4">
+    <row r="16" spans="1:10" ht="15">
       <c r="A16" s="59"/>
       <c r="B16" s="5">
         <v>8</v>
@@ -10346,7 +10373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="14.4">
+    <row r="17" spans="1:10" ht="15">
       <c r="A17" s="58" t="s">
         <v>19</v>
       </c>
@@ -10358,7 +10385,7 @@
       <c r="E17" s="12"/>
       <c r="F17" s="12"/>
     </row>
-    <row r="18" spans="1:10" ht="14.4">
+    <row r="18" spans="1:10" ht="15">
       <c r="A18" s="59"/>
       <c r="B18" s="5">
         <v>11</v>
@@ -10386,7 +10413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="28.8">
+    <row r="19" spans="1:10" ht="30">
       <c r="A19" s="59"/>
       <c r="B19" s="5">
         <v>13</v>
@@ -10398,7 +10425,7 @@
       <c r="E19" s="8"/>
       <c r="F19" s="8"/>
     </row>
-    <row r="20" spans="1:10" ht="28.8">
+    <row r="20" spans="1:10" ht="30">
       <c r="A20" s="59"/>
       <c r="B20" s="5">
         <v>14</v>
@@ -10410,7 +10437,7 @@
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
     </row>
-    <row r="21" spans="1:10" ht="14.4">
+    <row r="21" spans="1:10" ht="15">
       <c r="A21" s="59"/>
       <c r="B21" s="5">
         <v>15</v>
@@ -10422,7 +10449,7 @@
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
     </row>
-    <row r="22" spans="1:10" ht="14.4">
+    <row r="22" spans="1:10" ht="15">
       <c r="A22" s="59"/>
       <c r="B22" s="5">
         <v>16</v>
@@ -10434,7 +10461,7 @@
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
     </row>
-    <row r="23" spans="1:10" ht="14.4">
+    <row r="23" spans="1:10" ht="15">
       <c r="A23" s="58" t="s">
         <v>20</v>
       </c>
@@ -10446,7 +10473,7 @@
       <c r="E23" s="12"/>
       <c r="F23" s="12"/>
     </row>
-    <row r="24" spans="1:10" ht="28.8">
+    <row r="24" spans="1:10" ht="30">
       <c r="A24" s="59"/>
       <c r="B24" s="20">
         <v>17</v>
@@ -10474,7 +10501,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="28.8">
+    <row r="25" spans="1:10" ht="30">
       <c r="A25" s="59"/>
       <c r="B25" s="5">
         <v>18</v>
@@ -10486,7 +10513,7 @@
       <c r="E25" s="8"/>
       <c r="F25" s="8"/>
     </row>
-    <row r="26" spans="1:10" ht="14.4">
+    <row r="26" spans="1:10" ht="15">
       <c r="A26" s="59"/>
       <c r="B26" s="5">
         <v>19</v>
@@ -10498,7 +10525,7 @@
       <c r="E26" s="8"/>
       <c r="F26" s="8"/>
     </row>
-    <row r="27" spans="1:10" ht="14.4">
+    <row r="27" spans="1:10" ht="15">
       <c r="A27" s="59"/>
       <c r="B27" s="5">
         <v>21</v>
@@ -10510,7 +10537,7 @@
       <c r="E27" s="8"/>
       <c r="F27" s="8"/>
     </row>
-    <row r="28" spans="1:10" ht="14.4">
+    <row r="28" spans="1:10" ht="15">
       <c r="A28" s="59"/>
       <c r="B28" s="5">
         <v>22</v>
@@ -10522,7 +10549,7 @@
       <c r="E28" s="8"/>
       <c r="F28" s="8"/>
     </row>
-    <row r="29" spans="1:10" ht="14.4">
+    <row r="29" spans="1:10" ht="15">
       <c r="A29" s="60" t="s">
         <v>11</v>
       </c>
@@ -10534,7 +10561,7 @@
       <c r="E29" s="12"/>
       <c r="F29" s="12"/>
     </row>
-    <row r="30" spans="1:10" ht="14.4">
+    <row r="30" spans="1:10" ht="15">
       <c r="A30" s="60"/>
       <c r="B30" s="5">
         <v>24</v>
@@ -10562,7 +10589,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="28.8">
+    <row r="31" spans="1:10" ht="30">
       <c r="A31" s="60"/>
       <c r="B31" s="5">
         <v>26</v>
@@ -10574,7 +10601,7 @@
       <c r="E31" s="8"/>
       <c r="F31" s="8"/>
     </row>
-    <row r="32" spans="1:10" ht="14.4">
+    <row r="32" spans="1:10" ht="15">
       <c r="A32" s="60"/>
       <c r="B32" s="5">
         <v>27</v>
@@ -10586,7 +10613,7 @@
       <c r="E32" s="8"/>
       <c r="F32" s="8"/>
     </row>
-    <row r="33" spans="1:10" ht="14.4">
+    <row r="33" spans="1:10" ht="15">
       <c r="A33" s="60"/>
       <c r="B33" s="5">
         <v>28</v>
@@ -10598,7 +10625,7 @@
       <c r="E33" s="8"/>
       <c r="F33" s="8"/>
     </row>
-    <row r="34" spans="1:10" ht="14.4">
+    <row r="34" spans="1:10" ht="15">
       <c r="A34" s="60"/>
       <c r="B34" s="5">
         <v>29</v>
@@ -10622,7 +10649,7 @@
       <c r="E35" s="12"/>
       <c r="F35" s="12"/>
     </row>
-    <row r="36" spans="1:10" ht="28.8">
+    <row r="36" spans="1:10" ht="30">
       <c r="A36" s="57"/>
       <c r="B36" s="5">
         <v>30</v>
@@ -10650,7 +10677,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="14.4">
+    <row r="37" spans="1:10" ht="15">
       <c r="A37" s="57"/>
       <c r="B37" s="5">
         <v>31</v>
@@ -10662,7 +10689,7 @@
       <c r="E37" s="8"/>
       <c r="F37" s="8"/>
     </row>
-    <row r="38" spans="1:10" ht="28.8">
+    <row r="38" spans="1:10" ht="30">
       <c r="A38" s="57"/>
       <c r="B38" s="5">
         <v>32</v>
@@ -10674,7 +10701,7 @@
       <c r="E38" s="8"/>
       <c r="F38" s="8"/>
     </row>
-    <row r="39" spans="1:10" ht="14.4">
+    <row r="39" spans="1:10" ht="15">
       <c r="A39" s="57"/>
       <c r="B39" s="5"/>
       <c r="C39" s="8" t="s">
@@ -10684,7 +10711,7 @@
       <c r="E39" s="8"/>
       <c r="F39" s="8"/>
     </row>
-    <row r="40" spans="1:10" ht="14.4">
+    <row r="40" spans="1:10" ht="15">
       <c r="A40" s="57"/>
       <c r="B40" s="9"/>
       <c r="C40" s="10" t="s">
@@ -10694,7 +10721,7 @@
       <c r="E40" s="12"/>
       <c r="F40" s="12"/>
     </row>
-    <row r="41" spans="1:10" ht="14.4">
+    <row r="41" spans="1:10" ht="15">
       <c r="A41" s="57"/>
       <c r="B41" s="5">
         <v>33</v>
@@ -10722,7 +10749,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:10" ht="14.4">
+    <row r="42" spans="1:10" ht="15">
       <c r="A42" s="57"/>
       <c r="B42" s="5">
         <v>34</v>
@@ -10734,47 +10761,47 @@
       <c r="E42" s="8"/>
       <c r="F42" s="8"/>
     </row>
-    <row r="51" spans="2:3" ht="14.4">
+    <row r="51" spans="2:3" ht="15">
       <c r="B51"/>
       <c r="C51"/>
     </row>
-    <row r="52" spans="2:3" ht="14.4">
+    <row r="52" spans="2:3" ht="15">
       <c r="B52"/>
       <c r="C52"/>
     </row>
-    <row r="53" spans="2:3" ht="14.4">
+    <row r="53" spans="2:3" ht="15">
       <c r="B53"/>
       <c r="C53"/>
     </row>
-    <row r="54" spans="2:3" ht="14.4">
+    <row r="54" spans="2:3" ht="15">
       <c r="B54"/>
       <c r="C54"/>
     </row>
-    <row r="55" spans="2:3" ht="14.4">
+    <row r="55" spans="2:3" ht="15">
       <c r="B55"/>
       <c r="C55"/>
     </row>
-    <row r="56" spans="2:3" ht="14.4">
+    <row r="56" spans="2:3" ht="15">
       <c r="B56"/>
       <c r="C56"/>
     </row>
-    <row r="57" spans="2:3" ht="14.4">
+    <row r="57" spans="2:3" ht="15">
       <c r="B57"/>
       <c r="C57"/>
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="D3:F3"/>
     <mergeCell ref="A5:A14"/>
     <mergeCell ref="A15:A16"/>
     <mergeCell ref="A17:A22"/>
     <mergeCell ref="A29:A34"/>
     <mergeCell ref="A35:A42"/>
     <mergeCell ref="A23:A28"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="D3:F3"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D23 D15 D17 D40 D35 D29" xr:uid="{00000000-0002-0000-0300-000000000000}">
@@ -10792,14 +10819,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:J58"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="1" max="1" width="21.109375" customWidth="1"/>
-    <col min="2" max="2" width="5.33203125" style="4" customWidth="1"/>
-    <col min="3" max="3" width="71.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="29.6640625" customWidth="1"/>
-    <col min="6" max="6" width="32.6640625" customWidth="1"/>
+    <col min="1" max="1" width="21.140625" customWidth="1"/>
+    <col min="2" max="2" width="5.28515625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="71.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.7109375" customWidth="1"/>
+    <col min="6" max="6" width="32.7109375" customWidth="1"/>
     <col min="7" max="10" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -10828,7 +10855,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="15" thickBot="1">
+    <row r="3" spans="1:10" ht="15.75" thickBot="1">
       <c r="A3" s="62" t="s">
         <v>26</v>
       </c>
@@ -10840,7 +10867,7 @@
       <c r="E3" s="66"/>
       <c r="F3" s="67"/>
     </row>
-    <row r="4" spans="1:10" ht="14.4">
+    <row r="4" spans="1:10" ht="15">
       <c r="A4" s="6" t="s">
         <v>22</v>
       </c>
@@ -10872,7 +10899,7 @@
       <c r="E5" s="12"/>
       <c r="F5" s="12"/>
     </row>
-    <row r="6" spans="1:10" ht="14.4">
+    <row r="6" spans="1:10" ht="15">
       <c r="A6" s="59"/>
       <c r="B6" s="5">
         <v>1</v>
@@ -10900,7 +10927,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="14.4">
+    <row r="7" spans="1:10" ht="15">
       <c r="A7" s="59"/>
       <c r="B7" s="9"/>
       <c r="C7" s="10" t="s">
@@ -10910,7 +10937,7 @@
       <c r="E7" s="12"/>
       <c r="F7" s="12"/>
     </row>
-    <row r="8" spans="1:10" s="1" customFormat="1" ht="28.8">
+    <row r="8" spans="1:10" s="1" customFormat="1" ht="30">
       <c r="A8" s="59"/>
       <c r="B8" s="5">
         <v>2</v>
@@ -10938,7 +10965,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="14.4">
+    <row r="9" spans="1:10" ht="15">
       <c r="A9" s="59"/>
       <c r="B9" s="9"/>
       <c r="C9" s="10" t="s">
@@ -10948,7 +10975,7 @@
       <c r="E9" s="12"/>
       <c r="F9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="28.8">
+    <row r="10" spans="1:10" ht="30">
       <c r="A10" s="59"/>
       <c r="B10" s="5">
         <v>3</v>
@@ -10976,7 +11003,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="28.8">
+    <row r="11" spans="1:10" ht="30">
       <c r="A11" s="59"/>
       <c r="B11" s="5">
         <v>4</v>
@@ -11000,7 +11027,7 @@
       <c r="E12" s="8"/>
       <c r="F12" s="8"/>
     </row>
-    <row r="13" spans="1:10" ht="14.4">
+    <row r="13" spans="1:10" ht="15">
       <c r="A13" s="59"/>
       <c r="B13" s="9"/>
       <c r="C13" s="10" t="s">
@@ -11010,7 +11037,7 @@
       <c r="E13" s="12"/>
       <c r="F13" s="12"/>
     </row>
-    <row r="14" spans="1:10" ht="14.4">
+    <row r="14" spans="1:10" ht="15">
       <c r="A14" s="59"/>
       <c r="B14" s="5">
         <v>6</v>
@@ -11050,7 +11077,7 @@
       <c r="E15" s="12"/>
       <c r="F15" s="12"/>
     </row>
-    <row r="16" spans="1:10" ht="14.4">
+    <row r="16" spans="1:10" ht="15">
       <c r="A16" s="59"/>
       <c r="B16" s="5">
         <v>8</v>
@@ -11090,7 +11117,7 @@
       <c r="E17" s="12"/>
       <c r="F17" s="12"/>
     </row>
-    <row r="18" spans="1:10" ht="14.4">
+    <row r="18" spans="1:10" ht="30">
       <c r="A18" s="59"/>
       <c r="B18" s="5">
         <v>9</v>
@@ -11118,7 +11145,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="14.4">
+    <row r="19" spans="1:10" ht="15">
       <c r="A19" s="59"/>
       <c r="B19" s="5">
         <v>10</v>
@@ -11130,7 +11157,7 @@
       <c r="E19" s="8"/>
       <c r="F19" s="8"/>
     </row>
-    <row r="20" spans="1:10" ht="28.8">
+    <row r="20" spans="1:10" ht="30">
       <c r="A20" s="59"/>
       <c r="B20" s="5">
         <v>11</v>
@@ -11142,7 +11169,7 @@
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
     </row>
-    <row r="21" spans="1:10" ht="14.4">
+    <row r="21" spans="1:10" ht="15">
       <c r="A21" s="68"/>
       <c r="B21" s="5">
         <v>13</v>
@@ -11154,7 +11181,7 @@
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
     </row>
-    <row r="22" spans="1:10" ht="14.4">
+    <row r="22" spans="1:10" ht="15">
       <c r="A22" s="58" t="s">
         <v>20</v>
       </c>
@@ -11166,7 +11193,7 @@
       <c r="E22" s="12"/>
       <c r="F22" s="12"/>
     </row>
-    <row r="23" spans="1:10" ht="14.4">
+    <row r="23" spans="1:10" ht="15">
       <c r="A23" s="59"/>
       <c r="B23" s="5">
         <v>14</v>
@@ -11194,7 +11221,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="14.4">
+    <row r="24" spans="1:10" ht="15">
       <c r="A24" s="59"/>
       <c r="B24" s="5">
         <v>15</v>
@@ -11218,7 +11245,7 @@
       <c r="E25" s="12"/>
       <c r="F25" s="12"/>
     </row>
-    <row r="26" spans="1:10" s="1" customFormat="1" ht="28.8">
+    <row r="26" spans="1:10" s="1" customFormat="1" ht="30">
       <c r="A26" s="59"/>
       <c r="B26" s="20">
         <v>24</v>
@@ -11246,7 +11273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:10" s="1" customFormat="1" ht="43.2">
+    <row r="27" spans="1:10" s="1" customFormat="1" ht="45">
       <c r="A27" s="59"/>
       <c r="B27" s="5">
         <v>25</v>
@@ -11258,7 +11285,7 @@
       <c r="E27" s="8"/>
       <c r="F27" s="8"/>
     </row>
-    <row r="28" spans="1:10" ht="14.4">
+    <row r="28" spans="1:10" ht="15">
       <c r="A28" s="59"/>
       <c r="B28" s="9"/>
       <c r="C28" s="10" t="s">
@@ -11268,7 +11295,7 @@
       <c r="E28" s="12"/>
       <c r="F28" s="12"/>
     </row>
-    <row r="29" spans="1:10" ht="28.8">
+    <row r="29" spans="1:10" ht="30">
       <c r="A29" s="59"/>
       <c r="B29" s="20">
         <v>26</v>
@@ -11296,7 +11323,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="14.4">
+    <row r="30" spans="1:10" ht="15">
       <c r="A30" s="60" t="s">
         <v>11</v>
       </c>
@@ -11308,7 +11335,7 @@
       <c r="E30" s="12"/>
       <c r="F30" s="12"/>
     </row>
-    <row r="31" spans="1:10" ht="14.4">
+    <row r="31" spans="1:10" ht="15">
       <c r="A31" s="60"/>
       <c r="B31" s="5">
         <v>19</v>
@@ -11336,7 +11363,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="28.8">
+    <row r="32" spans="1:10" ht="30">
       <c r="A32" s="60"/>
       <c r="B32" s="5">
         <v>20</v>
@@ -11348,7 +11375,7 @@
       <c r="E32" s="8"/>
       <c r="F32" s="8"/>
     </row>
-    <row r="33" spans="1:10" ht="14.4">
+    <row r="33" spans="1:10" ht="15">
       <c r="A33" s="60"/>
       <c r="B33" s="5">
         <v>21</v>
@@ -11360,7 +11387,7 @@
       <c r="E33" s="8"/>
       <c r="F33" s="8"/>
     </row>
-    <row r="34" spans="1:10" ht="14.4">
+    <row r="34" spans="1:10" ht="15">
       <c r="A34" s="60"/>
       <c r="B34" s="5">
         <v>24</v>
@@ -11372,7 +11399,7 @@
       <c r="E34" s="8"/>
       <c r="F34" s="8"/>
     </row>
-    <row r="35" spans="1:10" ht="14.4">
+    <row r="35" spans="1:10" ht="15">
       <c r="A35" s="60"/>
       <c r="B35" s="5">
         <v>25</v>
@@ -11396,7 +11423,7 @@
       <c r="E36" s="12"/>
       <c r="F36" s="12"/>
     </row>
-    <row r="37" spans="1:10" ht="28.8">
+    <row r="37" spans="1:10" ht="30">
       <c r="A37" s="57"/>
       <c r="B37" s="5">
         <v>26</v>
@@ -11424,7 +11451,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="14.4">
+    <row r="38" spans="1:10" ht="15">
       <c r="A38" s="57"/>
       <c r="B38" s="5">
         <v>27</v>
@@ -11436,7 +11463,7 @@
       <c r="E38" s="8"/>
       <c r="F38" s="8"/>
     </row>
-    <row r="39" spans="1:10" ht="28.8">
+    <row r="39" spans="1:10" ht="30">
       <c r="A39" s="57"/>
       <c r="B39" s="5">
         <v>28</v>
@@ -11448,7 +11475,7 @@
       <c r="E39" s="8"/>
       <c r="F39" s="8"/>
     </row>
-    <row r="40" spans="1:10" ht="14.4">
+    <row r="40" spans="1:10" ht="15">
       <c r="A40" s="57"/>
       <c r="B40" s="5"/>
       <c r="C40" s="8" t="s">
@@ -11458,7 +11485,7 @@
       <c r="E40" s="8"/>
       <c r="F40" s="8"/>
     </row>
-    <row r="41" spans="1:10" ht="14.4">
+    <row r="41" spans="1:10" ht="15">
       <c r="A41" s="57"/>
       <c r="B41" s="9"/>
       <c r="C41" s="10" t="s">
@@ -11468,7 +11495,7 @@
       <c r="E41" s="12"/>
       <c r="F41" s="12"/>
     </row>
-    <row r="42" spans="1:10" ht="14.4">
+    <row r="42" spans="1:10" ht="15">
       <c r="A42" s="57"/>
       <c r="B42" s="5">
         <v>29</v>
@@ -11496,7 +11523,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:10" ht="14.4">
+    <row r="43" spans="1:10" ht="15">
       <c r="A43" s="57"/>
       <c r="B43" s="5">
         <v>30</v>
@@ -11508,41 +11535,36 @@
       <c r="E43" s="8"/>
       <c r="F43" s="8"/>
     </row>
-    <row r="52" spans="2:3" ht="14.4">
+    <row r="52" spans="2:3" ht="15">
       <c r="B52"/>
       <c r="C52"/>
     </row>
-    <row r="53" spans="2:3" ht="14.4">
+    <row r="53" spans="2:3" ht="15">
       <c r="B53"/>
       <c r="C53"/>
     </row>
-    <row r="54" spans="2:3" ht="14.4">
+    <row r="54" spans="2:3" ht="15">
       <c r="B54"/>
       <c r="C54"/>
     </row>
-    <row r="55" spans="2:3" ht="14.4">
+    <row r="55" spans="2:3" ht="15">
       <c r="B55"/>
       <c r="C55"/>
     </row>
-    <row r="56" spans="2:3" ht="14.4">
+    <row r="56" spans="2:3" ht="15">
       <c r="B56"/>
       <c r="C56"/>
     </row>
-    <row r="57" spans="2:3" ht="14.4">
+    <row r="57" spans="2:3" ht="15">
       <c r="B57"/>
       <c r="C57"/>
     </row>
-    <row r="58" spans="2:3" ht="14.4">
+    <row r="58" spans="2:3" ht="15">
       <c r="B58"/>
       <c r="C58"/>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A22:A24"/>
-    <mergeCell ref="A30:A35"/>
-    <mergeCell ref="A36:A43"/>
-    <mergeCell ref="A17:A21"/>
-    <mergeCell ref="A25:A29"/>
     <mergeCell ref="A5:A14"/>
     <mergeCell ref="A15:A16"/>
     <mergeCell ref="A1:F1"/>
@@ -11550,6 +11572,11 @@
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="D3:F3"/>
+    <mergeCell ref="A22:A24"/>
+    <mergeCell ref="A30:A35"/>
+    <mergeCell ref="A36:A43"/>
+    <mergeCell ref="A17:A21"/>
+    <mergeCell ref="A25:A29"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D25 D17 D15 D22 D41 D36 D30 D28" xr:uid="{00000000-0002-0000-0400-000000000000}">

</xml_diff>

<commit_message>
Replaneja os sprints e deixa o Checklist para o professor
Ajustes da Iniciação (#21):

- PCP: a Iniciação, prevista para fechar em 11/09, só terminou em 26/09,
  com a apresentação da fase e os ajustes da issue #21. O sprint 2
  registra o atraso no Realizado; os sprints 3 a 7 andam duas semanas,
  até 04/12, com os mesmos produtos e a mesma capacidade.
- A reserva de calendário até 04/12 virou o sprint 7: notas da aba
  Entregas e o RI-06 da aba Riscos atualizados.
- Checklist: a aba Ver-Iniciação1 volta ao estado do template, em
  branco. Quem preenche é o professor.
</commit_message>
<xml_diff>
--- a/6.Gerenciamento de Projeto/CARREGAJA - Checklist de Projeto.xlsx
+++ b/6.Gerenciamento de Projeto/CARREGAJA - Checklist de Projeto.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{077A368B-FBA1-43EB-B3C8-DAD3BA2D068B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B10FDBE1-5024-4C05-929B-C2422D6F8954}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="960" yWindow="960" windowWidth="21600" windowHeight="11235" tabRatio="666" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="666" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Indicadores" sheetId="6" r:id="rId1"/>
@@ -713,7 +713,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="114">
   <si>
     <t>Ambiente</t>
   </si>
@@ -1055,45 +1055,6 @@
   </si>
   <si>
     <t>Foram realizados os testes de aceitação por parte do usuário final?</t>
-  </si>
-  <si>
-    <t>Henrique de Almeida Marangoni Inacio (Scrum Master)</t>
-  </si>
-  <si>
-    <t>Sim</t>
-  </si>
-  <si>
-    <t>NA</t>
-  </si>
-  <si>
-    <t>Aprovado pelo Product Owner, que atua como representante do cliente (RE-16).</t>
-  </si>
-  <si>
-    <t>O Glossário é a subseção 1.3 do Visão, onde o template o posiciona. O SpinOff não prevê template autônomo para ele.</t>
-  </si>
-  <si>
-    <t>26/09/2026</t>
-  </si>
-  <si>
-    <t>O Documento de Requisitos, não previsto no SpinOff, tem template próprio: 1.Requisitos/Template - Documento de Requisitos.dotx.</t>
-  </si>
-  <si>
-    <t>Visão reduzido a uma visão geral na versão 4.0, após a apresentação da Iniciação; o detalhamento passou ao Documento de Requisitos.</t>
-  </si>
-  <si>
-    <t>Modelo mantido em CARREGAJA - Modelos de Análise e Design.asta, no formato do Template - Modelos Analise e Design do SpinOff, com os dois atores, os doze casos de uso UC01–UC12, cada um com descrição, e as relações de inclusão.</t>
-  </si>
-  <si>
-    <t>Protótipo não produzido: é saída de Detalhar Requisitos, da Elaboração.</t>
-  </si>
-  <si>
-    <t>Não houve reunião de levantamento a registrar: o projeto não dispõe de cliente externo (RE-16).</t>
-  </si>
-  <si>
-    <t>Não se aplica pelo mesmo motivo do item 16 (RE-16).</t>
-  </si>
-  <si>
-    <t>Plano de entregas com 7 sprints, o número calculado na aba Planejamento da PCP (6,13, arredondado para cima).</t>
   </si>
 </sst>
 </file>
@@ -1724,7 +1685,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -1956,19 +1917,19 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.8</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
@@ -1980,10 +1941,10 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>0</c:v>
@@ -2301,7 +2262,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.2</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -2310,7 +2271,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
@@ -7455,9 +7416,9 @@
       <c r="A3" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="B3" s="18">
+      <c r="B3" s="18" t="e">
         <f>'Ver-Iniciação1'!$F$2</f>
-        <v>1</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -7550,21 +7511,21 @@
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="22">
+      <c r="B2" s="22" t="e">
         <f>('Ver-Iniciação1'!$G$5/SUM('Ver-Iniciação1'!$G$5:'Ver-Iniciação1'!$J$5))</f>
-        <v>1</v>
-      </c>
-      <c r="C2" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="C2" s="22" t="e">
         <f>('Ver-Iniciação1'!$H$5/SUM('Ver-Iniciação1'!$G$5:'Ver-Iniciação1'!$J$5))</f>
-        <v>0</v>
-      </c>
-      <c r="D2" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D2" s="22" t="e">
         <f>('Ver-Iniciação1'!$I$5/SUM('Ver-Iniciação1'!$G$5:'Ver-Iniciação1'!$J$5))</f>
-        <v>0</v>
-      </c>
-      <c r="E2" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E2" s="22" t="e">
         <f>('Ver-Iniciação1'!$J$5/SUM('Ver-Iniciação1'!$G$5:'Ver-Iniciação1'!$J$5))</f>
-        <v>0</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="N2" t="s">
         <v>2</v>
@@ -7590,21 +7551,21 @@
       <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="22">
+      <c r="B3" s="22" t="e">
         <f>('Ver-Iniciação1'!$G$7/SUM('Ver-Iniciação1'!$G$7:'Ver-Iniciação1'!$J$7))</f>
-        <v>1</v>
-      </c>
-      <c r="C3" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="C3" s="22" t="e">
         <f>('Ver-Iniciação1'!$H$7/SUM('Ver-Iniciação1'!$G$7:'Ver-Iniciação1'!$J$7))</f>
-        <v>0</v>
-      </c>
-      <c r="D3" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D3" s="22" t="e">
         <f>('Ver-Iniciação1'!$I$7/SUM('Ver-Iniciação1'!$G$7:'Ver-Iniciação1'!$J$7))</f>
-        <v>0</v>
-      </c>
-      <c r="E3" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E3" s="22" t="e">
         <f>('Ver-Iniciação1'!$J$7/SUM('Ver-Iniciação1'!$G$7:'Ver-Iniciação1'!$J$7))</f>
-        <v>0</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="N3" t="s">
         <v>3</v>
@@ -7630,21 +7591,21 @@
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="22">
+      <c r="B4" s="22" t="e">
         <f>('Ver-Iniciação1'!$G$13/SUM('Ver-Iniciação1'!$G$13:'Ver-Iniciação1'!$J$13))</f>
-        <v>0.8</v>
-      </c>
-      <c r="C4" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="C4" s="22" t="e">
         <f>('Ver-Iniciação1'!$H$13/SUM('Ver-Iniciação1'!$G$13:'Ver-Iniciação1'!$J$13))</f>
-        <v>0</v>
-      </c>
-      <c r="D4" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D4" s="22" t="e">
         <f>('Ver-Iniciação1'!$I$13/SUM('Ver-Iniciação1'!$G$13:'Ver-Iniciação1'!$J$13))</f>
-        <v>0</v>
-      </c>
-      <c r="E4" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E4" s="22" t="e">
         <f>('Ver-Iniciação1'!$J$13/SUM('Ver-Iniciação1'!$G$13:'Ver-Iniciação1'!$J$13))</f>
-        <v>0.2</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="N4" t="s">
         <v>14</v>
@@ -7670,21 +7631,21 @@
       <c r="A5" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="22">
+      <c r="B5" s="22" t="e">
         <f>('Ver-Iniciação1'!$G$19/SUM('Ver-Iniciação1'!$G$19:'Ver-Iniciação1'!$J$19))</f>
-        <v>1</v>
-      </c>
-      <c r="C5" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="C5" s="22" t="e">
         <f>('Ver-Iniciação1'!$H$19/SUM('Ver-Iniciação1'!$G$19:'Ver-Iniciação1'!$J$19))</f>
-        <v>0</v>
-      </c>
-      <c r="D5" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D5" s="22" t="e">
         <f>('Ver-Iniciação1'!$I$19/SUM('Ver-Iniciação1'!$G$19:'Ver-Iniciação1'!$J$19))</f>
-        <v>0</v>
-      </c>
-      <c r="E5" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E5" s="22" t="e">
         <f>('Ver-Iniciação1'!$J$19/SUM('Ver-Iniciação1'!$G$19:'Ver-Iniciação1'!$J$19))</f>
-        <v>0</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="N5" t="s">
         <v>4</v>
@@ -7710,21 +7671,21 @@
       <c r="A6" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="22">
+      <c r="B6" s="22" t="e">
         <f>('Ver-Iniciação1'!$G$22/SUM('Ver-Iniciação1'!$G$22:'Ver-Iniciação1'!$J$22))</f>
-        <v>1</v>
-      </c>
-      <c r="C6" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="C6" s="22" t="e">
         <f>('Ver-Iniciação1'!$H$22/SUM('Ver-Iniciação1'!$G$22:'Ver-Iniciação1'!$J$22))</f>
-        <v>0</v>
-      </c>
-      <c r="D6" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D6" s="22" t="e">
         <f>('Ver-Iniciação1'!$I$22/SUM('Ver-Iniciação1'!$G$22:'Ver-Iniciação1'!$J$22))</f>
-        <v>0</v>
-      </c>
-      <c r="E6" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E6" s="22" t="e">
         <f>('Ver-Iniciação1'!$J$22/SUM('Ver-Iniciação1'!$G$22:'Ver-Iniciação1'!$J$22))</f>
-        <v>0</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="N6" t="s">
         <v>36</v>
@@ -7750,21 +7711,21 @@
       <c r="A7" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="22">
+      <c r="B7" s="22" t="e">
         <f>('Ver-Iniciação1'!$G$25/SUM('Ver-Iniciação1'!$G$25:'Ver-Iniciação1'!$J$25))</f>
-        <v>0</v>
-      </c>
-      <c r="C7" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="C7" s="22" t="e">
         <f>('Ver-Iniciação1'!$H$25/SUM('Ver-Iniciação1'!$G$25:'Ver-Iniciação1'!$J$25))</f>
-        <v>0</v>
-      </c>
-      <c r="D7" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D7" s="22" t="e">
         <f>('Ver-Iniciação1'!$I$25/SUM('Ver-Iniciação1'!$G$25:'Ver-Iniciação1'!$J$25))</f>
-        <v>0</v>
-      </c>
-      <c r="E7" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E7" s="22" t="e">
         <f>('Ver-Iniciação1'!$J$25/SUM('Ver-Iniciação1'!$G$25:'Ver-Iniciação1'!$J$25))</f>
-        <v>1</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="N7" t="s">
         <v>5</v>
@@ -7870,21 +7831,21 @@
       <c r="A10" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="22">
+      <c r="B10" s="22" t="e">
         <f>('Ver-Iniciação1'!$G$28/SUM('Ver-Iniciação1'!$G$28:'Ver-Iniciação1'!$J$28))</f>
-        <v>1</v>
-      </c>
-      <c r="C10" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="C10" s="22" t="e">
         <f>('Ver-Iniciação1'!$H$28/SUM('Ver-Iniciação1'!$G$28:'Ver-Iniciação1'!$J$28))</f>
-        <v>0</v>
-      </c>
-      <c r="D10" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D10" s="22" t="e">
         <f>('Ver-Iniciação1'!$I$28/SUM('Ver-Iniciação1'!$G$28:'Ver-Iniciação1'!$J$28))</f>
-        <v>0</v>
-      </c>
-      <c r="E10" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E10" s="22" t="e">
         <f>('Ver-Iniciação1'!$J$28/SUM('Ver-Iniciação1'!$G$28:'Ver-Iniciação1'!$J$28))</f>
-        <v>0</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="N10" t="s">
         <v>13</v>
@@ -7910,21 +7871,21 @@
       <c r="A11" t="s">
         <v>56</v>
       </c>
-      <c r="B11" s="22">
+      <c r="B11" s="22" t="e">
         <f>('Ver-Iniciação1'!$G$37/SUM('Ver-Iniciação1'!$G$37:'Ver-Iniciação1'!$J$37))</f>
-        <v>1</v>
-      </c>
-      <c r="C11" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="C11" s="22" t="e">
         <f>('Ver-Iniciação1'!$H$37/SUM('Ver-Iniciação1'!$G$37:'Ver-Iniciação1'!$J$37))</f>
-        <v>0</v>
-      </c>
-      <c r="D11" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D11" s="22" t="e">
         <f>('Ver-Iniciação1'!$I$37/SUM('Ver-Iniciação1'!$G$37:'Ver-Iniciação1'!$J$37))</f>
-        <v>0</v>
-      </c>
-      <c r="E11" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E11" s="22" t="e">
         <f>('Ver-Iniciação1'!$J$37/SUM('Ver-Iniciação1'!$G$37:'Ver-Iniciação1'!$J$37))</f>
-        <v>0</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="N11" t="s">
         <v>56</v>
@@ -8566,16 +8527,14 @@
         <v>25</v>
       </c>
       <c r="B2" s="47"/>
-      <c r="C2" s="40" t="s">
-        <v>119</v>
-      </c>
+      <c r="C2" s="40"/>
       <c r="D2" s="53" t="s">
         <v>44</v>
       </c>
       <c r="E2" s="54"/>
-      <c r="F2" s="42">
+      <c r="F2" s="42" t="e">
         <f>COUNTIF(D5:D41,"Sim")/(COUNTA(D5:D41)-COUNTIF(D5:D41,"NA"))</f>
-        <v>1</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="G2" s="39"/>
       <c r="H2" s="39"/>
@@ -8587,9 +8546,7 @@
         <v>26</v>
       </c>
       <c r="B3" s="47"/>
-      <c r="C3" s="41" t="s">
-        <v>114</v>
-      </c>
+      <c r="C3" s="41"/>
       <c r="D3" s="50" t="s">
         <v>43</v>
       </c>
@@ -8637,7 +8594,7 @@
       <c r="F5" s="31"/>
       <c r="G5" s="28">
         <f>COUNTIF(D6,"Sim")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H5" s="28">
         <f>COUNTIF(D6,"Parcialmente")</f>
@@ -8652,7 +8609,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="60">
+    <row r="6" spans="1:10" ht="15">
       <c r="A6" s="49"/>
       <c r="B6" s="32">
         <v>1</v>
@@ -8660,13 +8617,9 @@
       <c r="C6" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="D6" s="34" t="s">
-        <v>115</v>
-      </c>
+      <c r="D6" s="34"/>
       <c r="E6" s="33"/>
-      <c r="F6" s="33" t="s">
-        <v>120</v>
-      </c>
+      <c r="F6" s="33"/>
       <c r="G6" s="28"/>
       <c r="H6" s="28"/>
       <c r="I6" s="28"/>
@@ -8685,7 +8638,7 @@
       <c r="F7" s="31"/>
       <c r="G7" s="28">
         <f>COUNTIF(D8:D12,"Sim")</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H7" s="28">
         <f>COUNTIF(D8:D12,"Parcialmente")</f>
@@ -8708,9 +8661,7 @@
       <c r="C8" s="36" t="s">
         <v>72</v>
       </c>
-      <c r="D8" s="34" t="s">
-        <v>115</v>
-      </c>
+      <c r="D8" s="34"/>
       <c r="E8" s="33"/>
       <c r="F8" s="33"/>
       <c r="G8" s="28"/>
@@ -8726,9 +8677,7 @@
       <c r="C9" s="33" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="34" t="s">
-        <v>115</v>
-      </c>
+      <c r="D9" s="34"/>
       <c r="E9" s="33"/>
       <c r="F9" s="33"/>
       <c r="G9" s="28"/>
@@ -8744,9 +8693,7 @@
       <c r="C10" s="33" t="s">
         <v>77</v>
       </c>
-      <c r="D10" s="34" t="s">
-        <v>115</v>
-      </c>
+      <c r="D10" s="34"/>
       <c r="E10" s="33"/>
       <c r="F10" s="33"/>
       <c r="G10" s="28"/>
@@ -8754,7 +8701,7 @@
       <c r="I10" s="28"/>
       <c r="J10" s="28"/>
     </row>
-    <row r="11" spans="1:10" s="1" customFormat="1" ht="45">
+    <row r="11" spans="1:10" s="1" customFormat="1" ht="15">
       <c r="A11" s="45"/>
       <c r="B11" s="32">
         <v>5</v>
@@ -8762,13 +8709,9 @@
       <c r="C11" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="34" t="s">
-        <v>115</v>
-      </c>
+      <c r="D11" s="34"/>
       <c r="E11" s="33"/>
-      <c r="F11" s="33" t="s">
-        <v>121</v>
-      </c>
+      <c r="F11" s="33"/>
       <c r="G11" s="37"/>
       <c r="H11" s="37"/>
       <c r="I11" s="37"/>
@@ -8782,9 +8725,7 @@
       <c r="C12" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="D12" s="34" t="s">
-        <v>115</v>
-      </c>
+      <c r="D12" s="34"/>
       <c r="E12" s="33"/>
       <c r="F12" s="33"/>
       <c r="G12" s="28"/>
@@ -8803,7 +8744,7 @@
       <c r="F13" s="31"/>
       <c r="G13" s="28">
         <f>COUNTIF(D14:D18,"Sim")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H13" s="28">
         <f>COUNTIF(D14:D18,"Parcialmente")</f>
@@ -8815,10 +8756,10 @@
       </c>
       <c r="J13" s="28">
         <f>COUNTIF(D14:D18,"NA")</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="30">
       <c r="A14" s="45"/>
       <c r="B14" s="38">
         <v>7</v>
@@ -8826,13 +8767,9 @@
       <c r="C14" s="36" t="s">
         <v>72</v>
       </c>
-      <c r="D14" s="34" t="s">
-        <v>115</v>
-      </c>
+      <c r="D14" s="34"/>
       <c r="E14" s="33"/>
-      <c r="F14" s="33" t="s">
-        <v>122</v>
-      </c>
+      <c r="F14" s="33"/>
       <c r="G14" s="28"/>
       <c r="H14" s="28"/>
       <c r="I14" s="28"/>
@@ -8846,9 +8783,7 @@
       <c r="C15" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="D15" s="34" t="s">
-        <v>115</v>
-      </c>
+      <c r="D15" s="34"/>
       <c r="E15" s="33"/>
       <c r="F15" s="33"/>
       <c r="G15" s="37"/>
@@ -8864,9 +8799,7 @@
       <c r="C16" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="D16" s="34" t="s">
-        <v>115</v>
-      </c>
+      <c r="D16" s="34"/>
       <c r="E16" s="33"/>
       <c r="F16" s="33"/>
       <c r="G16" s="37"/>
@@ -8882,19 +8815,15 @@
       <c r="C17" s="36" t="s">
         <v>76</v>
       </c>
-      <c r="D17" s="34" t="s">
-        <v>116</v>
-      </c>
-      <c r="E17" s="33" t="s">
-        <v>123</v>
-      </c>
+      <c r="D17" s="34"/>
+      <c r="E17" s="33"/>
       <c r="F17" s="33"/>
       <c r="G17" s="37"/>
       <c r="H17" s="37"/>
       <c r="I17" s="37"/>
       <c r="J17" s="37"/>
     </row>
-    <row r="18" spans="1:10" s="1" customFormat="1" ht="30">
+    <row r="18" spans="1:10" s="1" customFormat="1" ht="15">
       <c r="A18" s="45"/>
       <c r="B18" s="32">
         <v>11</v>
@@ -8902,13 +8831,9 @@
       <c r="C18" s="33" t="s">
         <v>75</v>
       </c>
-      <c r="D18" s="34" t="s">
-        <v>115</v>
-      </c>
+      <c r="D18" s="34"/>
       <c r="E18" s="33"/>
-      <c r="F18" s="33" t="s">
-        <v>117</v>
-      </c>
+      <c r="F18" s="33"/>
       <c r="G18" s="37"/>
       <c r="H18" s="37"/>
       <c r="I18" s="37"/>
@@ -8925,7 +8850,7 @@
       <c r="F19" s="31"/>
       <c r="G19" s="28">
         <f>COUNTIF(D20:D21,"Sim")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H19" s="28">
         <f>COUNTIF(D20:D21,"Parcialmente")</f>
@@ -8948,9 +8873,7 @@
       <c r="C20" s="36" t="s">
         <v>78</v>
       </c>
-      <c r="D20" s="34" t="s">
-        <v>115</v>
-      </c>
+      <c r="D20" s="34"/>
       <c r="E20" s="33"/>
       <c r="F20" s="33"/>
       <c r="G20" s="28"/>
@@ -8966,9 +8889,7 @@
       <c r="C21" s="33" t="s">
         <v>80</v>
       </c>
-      <c r="D21" s="34" t="s">
-        <v>115</v>
-      </c>
+      <c r="D21" s="34"/>
       <c r="E21" s="33"/>
       <c r="F21" s="33"/>
       <c r="G21" s="28"/>
@@ -8987,7 +8908,7 @@
       <c r="F22" s="31"/>
       <c r="G22" s="28">
         <f>COUNTIF(D23:D24,"Sim")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H22" s="28">
         <f>COUNTIF(D23:D24,"Parcialmente")</f>
@@ -9002,7 +8923,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="45">
+    <row r="23" spans="1:10" ht="30">
       <c r="A23" s="45"/>
       <c r="B23" s="38">
         <v>14</v>
@@ -9010,13 +8931,9 @@
       <c r="C23" s="36" t="s">
         <v>72</v>
       </c>
-      <c r="D23" s="34" t="s">
-        <v>115</v>
-      </c>
+      <c r="D23" s="34"/>
       <c r="E23" s="33"/>
-      <c r="F23" s="33" t="s">
-        <v>118</v>
-      </c>
+      <c r="F23" s="33"/>
       <c r="G23" s="28"/>
       <c r="H23" s="28"/>
       <c r="I23" s="28"/>
@@ -9030,9 +8947,7 @@
       <c r="C24" s="33" t="s">
         <v>35</v>
       </c>
-      <c r="D24" s="34" t="s">
-        <v>115</v>
-      </c>
+      <c r="D24" s="34"/>
       <c r="E24" s="33"/>
       <c r="F24" s="33"/>
       <c r="G24" s="28"/>
@@ -9063,7 +8978,7 @@
       </c>
       <c r="J25" s="28">
         <f>COUNTIF(D26:D27,"NA")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:10" ht="30">
@@ -9074,19 +8989,15 @@
       <c r="C26" s="36" t="s">
         <v>72</v>
       </c>
-      <c r="D26" s="34" t="s">
-        <v>116</v>
-      </c>
-      <c r="E26" s="33" t="s">
-        <v>124</v>
-      </c>
+      <c r="D26" s="34"/>
+      <c r="E26" s="33"/>
       <c r="F26" s="33"/>
       <c r="G26" s="28"/>
       <c r="H26" s="28"/>
       <c r="I26" s="28"/>
       <c r="J26" s="28"/>
     </row>
-    <row r="27" spans="1:10" ht="30">
+    <row r="27" spans="1:10" ht="15">
       <c r="A27" s="45"/>
       <c r="B27" s="32">
         <v>17</v>
@@ -9094,12 +9005,8 @@
       <c r="C27" s="33" t="s">
         <v>37</v>
       </c>
-      <c r="D27" s="34" t="s">
-        <v>116</v>
-      </c>
-      <c r="E27" s="33" t="s">
-        <v>125</v>
-      </c>
+      <c r="D27" s="34"/>
+      <c r="E27" s="33"/>
       <c r="F27" s="33"/>
       <c r="G27" s="28"/>
       <c r="H27" s="28"/>
@@ -9117,7 +9024,7 @@
       <c r="F28" s="31"/>
       <c r="G28" s="28">
         <f>COUNTIF(D29:D36,"Sim")</f>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H28" s="28">
         <f>COUNTIF(D29:D36,"Parcialmente")</f>
@@ -9140,9 +9047,7 @@
       <c r="C29" s="36" t="s">
         <v>72</v>
       </c>
-      <c r="D29" s="34" t="s">
-        <v>115</v>
-      </c>
+      <c r="D29" s="34"/>
       <c r="E29" s="33"/>
       <c r="F29" s="33"/>
       <c r="G29" s="28"/>
@@ -9158,9 +9063,7 @@
       <c r="C30" s="33" t="s">
         <v>41</v>
       </c>
-      <c r="D30" s="34" t="s">
-        <v>115</v>
-      </c>
+      <c r="D30" s="34"/>
       <c r="E30" s="33"/>
       <c r="F30" s="33"/>
       <c r="G30" s="28"/>
@@ -9176,9 +9079,7 @@
       <c r="C31" s="33" t="s">
         <v>86</v>
       </c>
-      <c r="D31" s="34" t="s">
-        <v>115</v>
-      </c>
+      <c r="D31" s="34"/>
       <c r="E31" s="33"/>
       <c r="F31" s="33"/>
       <c r="G31" s="28"/>
@@ -9194,9 +9095,7 @@
       <c r="C32" s="33" t="s">
         <v>82</v>
       </c>
-      <c r="D32" s="34" t="s">
-        <v>115</v>
-      </c>
+      <c r="D32" s="34"/>
       <c r="E32" s="33"/>
       <c r="F32" s="33"/>
       <c r="G32" s="28"/>
@@ -9212,9 +9111,7 @@
       <c r="C33" s="33" t="s">
         <v>83</v>
       </c>
-      <c r="D33" s="34" t="s">
-        <v>115</v>
-      </c>
+      <c r="D33" s="34"/>
       <c r="E33" s="33"/>
       <c r="F33" s="33"/>
       <c r="G33" s="28"/>
@@ -9222,7 +9119,7 @@
       <c r="I33" s="28"/>
       <c r="J33" s="28"/>
     </row>
-    <row r="34" spans="1:10" ht="45">
+    <row r="34" spans="1:10" ht="30">
       <c r="A34" s="45"/>
       <c r="B34" s="32">
         <v>26</v>
@@ -9230,13 +9127,9 @@
       <c r="C34" s="33" t="s">
         <v>87</v>
       </c>
-      <c r="D34" s="34" t="s">
-        <v>115</v>
-      </c>
+      <c r="D34" s="34"/>
       <c r="E34" s="28"/>
-      <c r="F34" s="33" t="s">
-        <v>126</v>
-      </c>
+      <c r="F34" s="33"/>
       <c r="G34" s="28"/>
       <c r="H34" s="28"/>
       <c r="I34" s="28"/>
@@ -9250,9 +9143,7 @@
       <c r="C35" s="33" t="s">
         <v>84</v>
       </c>
-      <c r="D35" s="34" t="s">
-        <v>115</v>
-      </c>
+      <c r="D35" s="34"/>
       <c r="E35" s="33"/>
       <c r="F35" s="33"/>
       <c r="G35" s="28"/>
@@ -9260,7 +9151,7 @@
       <c r="I35" s="28"/>
       <c r="J35" s="28"/>
     </row>
-    <row r="36" spans="1:10" ht="30">
+    <row r="36" spans="1:10" ht="15">
       <c r="A36" s="45"/>
       <c r="B36" s="32">
         <v>28</v>
@@ -9268,13 +9159,9 @@
       <c r="C36" s="33" t="s">
         <v>85</v>
       </c>
-      <c r="D36" s="33" t="s">
-        <v>115</v>
-      </c>
+      <c r="D36" s="33"/>
       <c r="E36" s="33"/>
-      <c r="F36" s="33" t="s">
-        <v>117</v>
-      </c>
+      <c r="F36" s="33"/>
       <c r="G36" s="28"/>
       <c r="H36" s="28"/>
       <c r="I36" s="28"/>
@@ -9293,7 +9180,7 @@
       <c r="F37" s="31"/>
       <c r="G37" s="28">
         <f>COUNTIF(D38:D41,"Sim")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H37" s="28">
         <f>COUNTIF(D38:D41,"Parcialmente")</f>
@@ -9316,9 +9203,7 @@
       <c r="C38" s="36" t="s">
         <v>73</v>
       </c>
-      <c r="D38" s="34" t="s">
-        <v>115</v>
-      </c>
+      <c r="D38" s="34"/>
       <c r="E38" s="33"/>
       <c r="F38" s="33"/>
       <c r="G38" s="28"/>
@@ -9334,9 +9219,7 @@
       <c r="C39" s="33" t="s">
         <v>38</v>
       </c>
-      <c r="D39" s="34" t="s">
-        <v>115</v>
-      </c>
+      <c r="D39" s="34"/>
       <c r="E39" s="33"/>
       <c r="F39" s="33"/>
       <c r="G39" s="28"/>
@@ -9352,9 +9235,7 @@
       <c r="C40" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="D40" s="34" t="s">
-        <v>115</v>
-      </c>
+      <c r="D40" s="34"/>
       <c r="E40" s="33"/>
       <c r="F40" s="33"/>
       <c r="G40" s="28"/>
@@ -9370,9 +9251,7 @@
       <c r="C41" s="33" t="s">
         <v>42</v>
       </c>
-      <c r="D41" s="34" t="s">
-        <v>115</v>
-      </c>
+      <c r="D41" s="34"/>
       <c r="E41" s="33"/>
       <c r="F41" s="33"/>
       <c r="G41" s="28"/>
@@ -10791,17 +10670,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="D3:F3"/>
     <mergeCell ref="A5:A14"/>
     <mergeCell ref="A15:A16"/>
     <mergeCell ref="A17:A22"/>
     <mergeCell ref="A29:A34"/>
     <mergeCell ref="A35:A42"/>
     <mergeCell ref="A23:A28"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="D3:F3"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D23 D15 D17 D40 D35 D29" xr:uid="{00000000-0002-0000-0300-000000000000}">
@@ -11565,6 +11444,11 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A22:A24"/>
+    <mergeCell ref="A30:A35"/>
+    <mergeCell ref="A36:A43"/>
+    <mergeCell ref="A17:A21"/>
+    <mergeCell ref="A25:A29"/>
     <mergeCell ref="A5:A14"/>
     <mergeCell ref="A15:A16"/>
     <mergeCell ref="A1:F1"/>
@@ -11572,11 +11456,6 @@
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="D3:F3"/>
-    <mergeCell ref="A22:A24"/>
-    <mergeCell ref="A30:A35"/>
-    <mergeCell ref="A36:A43"/>
-    <mergeCell ref="A17:A21"/>
-    <mergeCell ref="A25:A29"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D25 D17 D15 D22 D41 D36 D30 D28" xr:uid="{00000000-0002-0000-0400-000000000000}">

</xml_diff>